<commit_message>
district heating partial data
</commit_message>
<xml_diff>
--- a/data/buses.xlsx
+++ b/data/buses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Geteilte Ablagen\KEKS- Kores\Code\Pypsa proto\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Keks-repo\KEKS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8752BEC0-F59C-49CA-B8E8-BEDD5AB8875B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9E9DD5-EAC3-4413-9791-99016CF778F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3015" yWindow="1590" windowWidth="21600" windowHeight="13185" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
   <si>
     <t>name</t>
   </si>
@@ -61,6 +61,15 @@
   </si>
   <si>
     <t>MV_bus_2</t>
+  </si>
+  <si>
+    <t>Residential_2</t>
+  </si>
+  <si>
+    <t>Residential_3</t>
+  </si>
+  <si>
+    <t>DEP_1</t>
   </si>
 </sst>
 </file>
@@ -378,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -504,6 +513,57 @@
         <v>6</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <v>0.4</v>
+      </c>
+      <c r="C8">
+        <v>7.9462320000000002</v>
+      </c>
+      <c r="D8">
+        <v>48.466816999999999</v>
+      </c>
+      <c r="E8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9">
+        <v>0.4</v>
+      </c>
+      <c r="C9">
+        <v>7.9479110000000004</v>
+      </c>
+      <c r="D9">
+        <v>48.465905999999997</v>
+      </c>
+      <c r="E9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10">
+        <v>0.4</v>
+      </c>
+      <c r="C10">
+        <v>7.9468259999999997</v>
+      </c>
+      <c r="D10">
+        <v>48.465688</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>